<commit_message>
New run of the Chuuchuu data to be sure cancelled trains are not dpouble counted in case of partial cancellation + delay
</commit_message>
<xml_diff>
--- a/summary_stats/chuuchuu_summary_2025_01.xlsx
+++ b/summary_stats/chuuchuu_summary_2025_01.xlsx
@@ -1454,13 +1454,13 @@
         <v>1</v>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O13" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P13" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q13" t="n">
         <v>23</v>
@@ -2007,25 +2007,25 @@
         <v>74</v>
       </c>
       <c r="N20" t="n">
-        <v>949</v>
+        <v>924</v>
       </c>
       <c r="O20" t="n">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="P20" t="n">
-        <v>759</v>
+        <v>734</v>
       </c>
       <c r="Q20" t="n">
-        <v>593</v>
+        <v>569</v>
       </c>
       <c r="R20" t="n">
-        <v>474</v>
+        <v>453</v>
       </c>
       <c r="S20" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="T20" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="U20" t="n">
         <v>1701</v>
@@ -2560,25 +2560,25 @@
         <v>339</v>
       </c>
       <c r="N27" t="n">
-        <v>1909</v>
+        <v>1787</v>
       </c>
       <c r="O27" t="n">
-        <v>1542</v>
+        <v>1435</v>
       </c>
       <c r="P27" t="n">
-        <v>1392</v>
+        <v>1290</v>
       </c>
       <c r="Q27" t="n">
-        <v>1005</v>
+        <v>929</v>
       </c>
       <c r="R27" t="n">
-        <v>722</v>
+        <v>662</v>
       </c>
       <c r="S27" t="n">
-        <v>321</v>
+        <v>284</v>
       </c>
       <c r="T27" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="U27" t="n">
         <v>4076</v>
@@ -2639,25 +2639,25 @@
         <v>101</v>
       </c>
       <c r="N28" t="n">
-        <v>657</v>
+        <v>629</v>
       </c>
       <c r="O28" t="n">
-        <v>517</v>
+        <v>491</v>
       </c>
       <c r="P28" t="n">
-        <v>470</v>
+        <v>444</v>
       </c>
       <c r="Q28" t="n">
-        <v>366</v>
+        <v>347</v>
       </c>
       <c r="R28" t="n">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="S28" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="T28" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="U28" t="n">
         <v>1634</v>
@@ -2718,25 +2718,25 @@
         <v>1100</v>
       </c>
       <c r="N29" t="n">
-        <v>6989</v>
+        <v>6604</v>
       </c>
       <c r="O29" t="n">
-        <v>5978</v>
+        <v>5617</v>
       </c>
       <c r="P29" t="n">
-        <v>5567</v>
+        <v>5219</v>
       </c>
       <c r="Q29" t="n">
-        <v>4333</v>
+        <v>4015</v>
       </c>
       <c r="R29" t="n">
-        <v>3297</v>
+        <v>3024</v>
       </c>
       <c r="S29" t="n">
-        <v>1662</v>
+        <v>1479</v>
       </c>
       <c r="T29" t="n">
-        <v>429</v>
+        <v>360</v>
       </c>
       <c r="U29" t="n">
         <v>13210</v>
@@ -2797,25 +2797,25 @@
         <v>203</v>
       </c>
       <c r="N30" t="n">
-        <v>1959</v>
+        <v>1881</v>
       </c>
       <c r="O30" t="n">
-        <v>1609</v>
+        <v>1538</v>
       </c>
       <c r="P30" t="n">
-        <v>1494</v>
+        <v>1425</v>
       </c>
       <c r="Q30" t="n">
-        <v>1166</v>
+        <v>1100</v>
       </c>
       <c r="R30" t="n">
-        <v>911</v>
+        <v>853</v>
       </c>
       <c r="S30" t="n">
-        <v>474</v>
+        <v>429</v>
       </c>
       <c r="T30" t="n">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="U30" t="n">
         <v>3326</v>
@@ -3113,25 +3113,25 @@
         <v>42</v>
       </c>
       <c r="N34" t="n">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="O34" t="n">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="P34" t="n">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="Q34" t="n">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="R34" t="n">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="S34" t="n">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="T34" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="U34" t="n">
         <v>564</v>
@@ -3192,25 +3192,25 @@
         <v>26</v>
       </c>
       <c r="N35" t="n">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="O35" t="n">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="P35" t="n">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="Q35" t="n">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="R35" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="S35" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="T35" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U35" t="n">
         <v>585</v>
@@ -3271,19 +3271,19 @@
         <v>16</v>
       </c>
       <c r="N36" t="n">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="O36" t="n">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="P36" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Q36" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="R36" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S36" t="n">
         <v>34</v>
@@ -4061,25 +4061,25 @@
         <v>306</v>
       </c>
       <c r="N46" t="n">
-        <v>857</v>
+        <v>775</v>
       </c>
       <c r="O46" t="n">
-        <v>846</v>
+        <v>764</v>
       </c>
       <c r="P46" t="n">
-        <v>841</v>
+        <v>760</v>
       </c>
       <c r="Q46" t="n">
-        <v>660</v>
+        <v>592</v>
       </c>
       <c r="R46" t="n">
-        <v>509</v>
+        <v>453</v>
       </c>
       <c r="S46" t="n">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="T46" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="U46" t="n">
         <v>2884</v>
@@ -4219,25 +4219,25 @@
         <v>31</v>
       </c>
       <c r="N48" t="n">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="O48" t="n">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="P48" t="n">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="Q48" t="n">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="R48" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="S48" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="T48" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="U48" t="n">
         <v>349</v>
@@ -4298,16 +4298,16 @@
         <v>1</v>
       </c>
       <c r="N49" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O49" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P49" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R49" t="n">
         <v>3</v>
@@ -5483,22 +5483,22 @@
         <v>4032</v>
       </c>
       <c r="N64" t="n">
-        <v>4646</v>
+        <v>4502</v>
       </c>
       <c r="O64" t="n">
-        <v>2464</v>
+        <v>2372</v>
       </c>
       <c r="P64" t="n">
-        <v>1951</v>
+        <v>1870</v>
       </c>
       <c r="Q64" t="n">
-        <v>953</v>
+        <v>900</v>
       </c>
       <c r="R64" t="n">
-        <v>416</v>
+        <v>387</v>
       </c>
       <c r="S64" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="T64" t="n">
         <v>4</v>
@@ -5562,19 +5562,19 @@
         <v>42</v>
       </c>
       <c r="N65" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="O65" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P65" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="Q65" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="R65" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="S65" t="n">
         <v>57</v>
@@ -5720,22 +5720,22 @@
         <v>931</v>
       </c>
       <c r="N67" t="n">
-        <v>508</v>
+        <v>440</v>
       </c>
       <c r="O67" t="n">
-        <v>328</v>
+        <v>281</v>
       </c>
       <c r="P67" t="n">
-        <v>276</v>
+        <v>229</v>
       </c>
       <c r="Q67" t="n">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="R67" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="S67" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T67" t="n">
         <v>1</v>
@@ -5878,22 +5878,22 @@
         <v>7</v>
       </c>
       <c r="N69" t="n">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="O69" t="n">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="P69" t="n">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="Q69" t="n">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="R69" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="S69" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="T69" t="n">
         <v>8</v>
@@ -6036,19 +6036,19 @@
         <v>5</v>
       </c>
       <c r="N71" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O71" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P71" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Q71" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="R71" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S71" t="n">
         <v>46</v>
@@ -6194,13 +6194,13 @@
         <v>50</v>
       </c>
       <c r="N73" t="n">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="O73" t="n">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="P73" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="Q73" t="n">
         <v>57</v>
@@ -6352,22 +6352,22 @@
         <v>3998</v>
       </c>
       <c r="N75" t="n">
-        <v>5630</v>
+        <v>5456</v>
       </c>
       <c r="O75" t="n">
-        <v>2665</v>
+        <v>2570</v>
       </c>
       <c r="P75" t="n">
-        <v>1981</v>
+        <v>1902</v>
       </c>
       <c r="Q75" t="n">
-        <v>817</v>
+        <v>782</v>
       </c>
       <c r="R75" t="n">
-        <v>317</v>
+        <v>304</v>
       </c>
       <c r="S75" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="T75" t="n">
         <v>0</v>
@@ -6431,19 +6431,19 @@
         <v>1124</v>
       </c>
       <c r="N76" t="n">
-        <v>3027</v>
+        <v>2956</v>
       </c>
       <c r="O76" t="n">
-        <v>1109</v>
+        <v>1070</v>
       </c>
       <c r="P76" t="n">
-        <v>757</v>
+        <v>728</v>
       </c>
       <c r="Q76" t="n">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="R76" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="S76" t="n">
         <v>8</v>
@@ -6826,16 +6826,16 @@
         <v>10</v>
       </c>
       <c r="N81" t="n">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="O81" t="n">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="P81" t="n">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="Q81" t="n">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="R81" t="n">
         <v>155</v>
@@ -7695,19 +7695,19 @@
         <v>59</v>
       </c>
       <c r="N92" t="n">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="O92" t="n">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="P92" t="n">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="Q92" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="R92" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S92" t="n">
         <v>26</v>
@@ -7774,25 +7774,25 @@
         <v>15</v>
       </c>
       <c r="N93" t="n">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="O93" t="n">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="P93" t="n">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="Q93" t="n">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="R93" t="n">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="S93" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="T93" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="U93" t="n">
         <v>1075</v>
@@ -7932,25 +7932,25 @@
         <v>55</v>
       </c>
       <c r="N95" t="n">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="O95" t="n">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="P95" t="n">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="Q95" t="n">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="R95" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="S95" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="T95" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="U95" t="n">
         <v>875</v>
@@ -8011,22 +8011,22 @@
         <v>13</v>
       </c>
       <c r="N96" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="O96" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="P96" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="Q96" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="R96" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="S96" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T96" t="n">
         <v>16</v>
@@ -8406,25 +8406,25 @@
         <v>20</v>
       </c>
       <c r="N101" t="n">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="O101" t="n">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="P101" t="n">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="Q101" t="n">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="R101" t="n">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="S101" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="T101" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="U101" t="n">
         <v>1319</v>
@@ -9433,22 +9433,22 @@
         <v>57</v>
       </c>
       <c r="N114" t="n">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="O114" t="n">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="P114" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="Q114" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="R114" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S114" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="T114" t="n">
         <v>6</v>
@@ -10065,16 +10065,16 @@
         <v>114</v>
       </c>
       <c r="N122" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O122" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="P122" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="Q122" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="R122" t="n">
         <v>13</v>
@@ -10381,7 +10381,7 @@
         <v>141</v>
       </c>
       <c r="N126" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="O126" t="n">
         <v>150</v>
@@ -11566,16 +11566,16 @@
         <v>17</v>
       </c>
       <c r="N141" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="O141" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="P141" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q141" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="R141" t="n">
         <v>12</v>
@@ -11645,25 +11645,25 @@
         <v>591</v>
       </c>
       <c r="N142" t="n">
-        <v>5699</v>
+        <v>5630</v>
       </c>
       <c r="O142" t="n">
-        <v>3421</v>
+        <v>3366</v>
       </c>
       <c r="P142" t="n">
-        <v>2732</v>
+        <v>2682</v>
       </c>
       <c r="Q142" t="n">
-        <v>1258</v>
+        <v>1227</v>
       </c>
       <c r="R142" t="n">
-        <v>651</v>
+        <v>628</v>
       </c>
       <c r="S142" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="T142" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U142" t="n">
         <v>27977</v>
@@ -11882,19 +11882,19 @@
         <v>23</v>
       </c>
       <c r="N145" t="n">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="O145" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="P145" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="Q145" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="R145" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="S145" t="n">
         <v>19</v>
@@ -11961,19 +11961,19 @@
         <v>153</v>
       </c>
       <c r="N146" t="n">
-        <v>3093</v>
+        <v>3060</v>
       </c>
       <c r="O146" t="n">
-        <v>1671</v>
+        <v>1648</v>
       </c>
       <c r="P146" t="n">
-        <v>1299</v>
+        <v>1280</v>
       </c>
       <c r="Q146" t="n">
-        <v>509</v>
+        <v>499</v>
       </c>
       <c r="R146" t="n">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="S146" t="n">
         <v>39</v>
@@ -12040,13 +12040,13 @@
         <v>39</v>
       </c>
       <c r="N147" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O147" t="n">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="P147" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="Q147" t="n">
         <v>46</v>
@@ -12277,22 +12277,22 @@
         <v>76</v>
       </c>
       <c r="N150" t="n">
-        <v>1146</v>
+        <v>1143</v>
       </c>
       <c r="O150" t="n">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="P150" t="n">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="Q150" t="n">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="R150" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="S150" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T150" t="n">
         <v>2</v>
@@ -12356,7 +12356,7 @@
         <v>7</v>
       </c>
       <c r="N151" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O151" t="n">
         <v>14</v>
@@ -12435,25 +12435,25 @@
         <v>374</v>
       </c>
       <c r="N152" t="n">
-        <v>3840</v>
+        <v>3786</v>
       </c>
       <c r="O152" t="n">
-        <v>2091</v>
+        <v>2059</v>
       </c>
       <c r="P152" t="n">
-        <v>1620</v>
+        <v>1595</v>
       </c>
       <c r="Q152" t="n">
-        <v>689</v>
+        <v>675</v>
       </c>
       <c r="R152" t="n">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="S152" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="T152" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U152" t="n">
         <v>27838</v>
@@ -12514,19 +12514,19 @@
         <v>100</v>
       </c>
       <c r="N153" t="n">
-        <v>546</v>
+        <v>537</v>
       </c>
       <c r="O153" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="P153" t="n">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="Q153" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="R153" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S153" t="n">
         <v>11</v>
@@ -12830,22 +12830,22 @@
         <v>39</v>
       </c>
       <c r="N157" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="O157" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="P157" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="Q157" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="R157" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="S157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T157" t="n">
         <v>0</v>
@@ -13146,25 +13146,25 @@
         <v>60</v>
       </c>
       <c r="N161" t="n">
-        <v>543</v>
+        <v>527</v>
       </c>
       <c r="O161" t="n">
-        <v>367</v>
+        <v>353</v>
       </c>
       <c r="P161" t="n">
-        <v>367</v>
+        <v>353</v>
       </c>
       <c r="Q161" t="n">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="R161" t="n">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="S161" t="n">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="T161" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="U161" t="n">
         <v>1652</v>
@@ -13462,19 +13462,19 @@
         <v>1</v>
       </c>
       <c r="N165" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O165" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P165" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q165" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R165" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S165" t="n">
         <v>4</v>
@@ -13857,25 +13857,25 @@
         <v>143</v>
       </c>
       <c r="N170" t="n">
-        <v>2866</v>
+        <v>2819</v>
       </c>
       <c r="O170" t="n">
-        <v>1720</v>
+        <v>1679</v>
       </c>
       <c r="P170" t="n">
-        <v>1720</v>
+        <v>1679</v>
       </c>
       <c r="Q170" t="n">
-        <v>1201</v>
+        <v>1163</v>
       </c>
       <c r="R170" t="n">
-        <v>916</v>
+        <v>880</v>
       </c>
       <c r="S170" t="n">
-        <v>453</v>
+        <v>425</v>
       </c>
       <c r="T170" t="n">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="U170" t="n">
         <v>10824</v>
@@ -13936,22 +13936,22 @@
         <v>2</v>
       </c>
       <c r="N171" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="O171" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P171" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q171" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="R171" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S171" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T171" t="n">
         <v>12</v>
@@ -14884,25 +14884,25 @@
         <v>19</v>
       </c>
       <c r="N183" t="n">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="O183" t="n">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="P183" t="n">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q183" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="R183" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="S183" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="T183" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U183" t="n">
         <v>495</v>
@@ -14963,22 +14963,22 @@
         <v>9</v>
       </c>
       <c r="N184" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O184" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P184" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Q184" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="R184" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="S184" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T184" t="n">
         <v>7</v>
@@ -15042,25 +15042,25 @@
         <v>176</v>
       </c>
       <c r="N185" t="n">
-        <v>2989</v>
+        <v>2974</v>
       </c>
       <c r="O185" t="n">
-        <v>2283</v>
+        <v>2268</v>
       </c>
       <c r="P185" t="n">
-        <v>2057</v>
+        <v>2042</v>
       </c>
       <c r="Q185" t="n">
-        <v>1453</v>
+        <v>1440</v>
       </c>
       <c r="R185" t="n">
-        <v>1071</v>
+        <v>1058</v>
       </c>
       <c r="S185" t="n">
-        <v>553</v>
+        <v>544</v>
       </c>
       <c r="T185" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="U185" t="n">
         <v>6934</v>
@@ -15200,25 +15200,25 @@
         <v>174</v>
       </c>
       <c r="N187" t="n">
-        <v>1283</v>
+        <v>1268</v>
       </c>
       <c r="O187" t="n">
-        <v>1018</v>
+        <v>1004</v>
       </c>
       <c r="P187" t="n">
-        <v>910</v>
+        <v>897</v>
       </c>
       <c r="Q187" t="n">
-        <v>608</v>
+        <v>597</v>
       </c>
       <c r="R187" t="n">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="S187" t="n">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="T187" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="U187" t="n">
         <v>3129</v>
@@ -15516,16 +15516,16 @@
         <v>327</v>
       </c>
       <c r="N191" t="n">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="O191" t="n">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="P191" t="n">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q191" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="R191" t="n">
         <v>52</v>
@@ -15832,22 +15832,22 @@
         <v>10</v>
       </c>
       <c r="N195" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="O195" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="P195" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="Q195" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R195" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="S195" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="T195" t="n">
         <v>4</v>
@@ -15911,25 +15911,25 @@
         <v>7820</v>
       </c>
       <c r="N196" t="n">
-        <v>42279</v>
+        <v>41819</v>
       </c>
       <c r="O196" t="n">
-        <v>23477</v>
+        <v>23134</v>
       </c>
       <c r="P196" t="n">
-        <v>18494</v>
+        <v>18185</v>
       </c>
       <c r="Q196" t="n">
-        <v>9176</v>
+        <v>8957</v>
       </c>
       <c r="R196" t="n">
-        <v>5310</v>
+        <v>5154</v>
       </c>
       <c r="S196" t="n">
-        <v>1693</v>
+        <v>1614</v>
       </c>
       <c r="T196" t="n">
-        <v>375</v>
+        <v>357</v>
       </c>
       <c r="U196" t="n">
         <v>217988</v>
@@ -15990,22 +15990,22 @@
         <v>334</v>
       </c>
       <c r="N197" t="n">
-        <v>1247</v>
+        <v>1243</v>
       </c>
       <c r="O197" t="n">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="P197" t="n">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="Q197" t="n">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="R197" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="S197" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="T197" t="n">
         <v>2</v>
@@ -17329,16 +17329,16 @@
         <v>3</v>
       </c>
       <c r="N214" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O214" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P214" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q214" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R214" t="n">
         <v>2</v>
@@ -17566,25 +17566,25 @@
         <v>10</v>
       </c>
       <c r="N217" t="n">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="O217" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="P217" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="Q217" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="R217" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="S217" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T217" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U217" t="n">
         <v>363</v>
@@ -18428,19 +18428,19 @@
         <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="R6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T6" t="n">
         <v>4</v>
@@ -18680,22 +18680,22 @@
         <v>39</v>
       </c>
       <c r="O9" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="P9" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="Q9" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="R9" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="S9" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="T9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -19016,25 +19016,25 @@
         <v>60</v>
       </c>
       <c r="O13" t="n">
-        <v>543</v>
+        <v>527</v>
       </c>
       <c r="P13" t="n">
-        <v>367</v>
+        <v>353</v>
       </c>
       <c r="Q13" t="n">
-        <v>367</v>
+        <v>353</v>
       </c>
       <c r="R13" t="n">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="S13" t="n">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="T13" t="n">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="U13" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="V13" t="n">
         <v>1652</v>
@@ -19352,25 +19352,25 @@
         <v>143</v>
       </c>
       <c r="O17" t="n">
-        <v>2866</v>
+        <v>2819</v>
       </c>
       <c r="P17" t="n">
-        <v>1720</v>
+        <v>1679</v>
       </c>
       <c r="Q17" t="n">
-        <v>1720</v>
+        <v>1679</v>
       </c>
       <c r="R17" t="n">
-        <v>1201</v>
+        <v>1163</v>
       </c>
       <c r="S17" t="n">
-        <v>916</v>
+        <v>880</v>
       </c>
       <c r="T17" t="n">
-        <v>453</v>
+        <v>425</v>
       </c>
       <c r="U17" t="n">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="V17" t="n">
         <v>10824</v>
@@ -19436,22 +19436,22 @@
         <v>2</v>
       </c>
       <c r="O18" t="n">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="P18" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q18" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="R18" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="S18" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="T18" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="U18" t="n">
         <v>12</v>
@@ -19898,22 +19898,22 @@
         <v>14</v>
       </c>
       <c r="O3" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="P3" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q3" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R3" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="S3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U3" t="n">
         <v>5</v>
@@ -20150,22 +20150,22 @@
         <v>4</v>
       </c>
       <c r="O6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="P6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U6" t="n">
         <v>1</v>
@@ -21410,25 +21410,25 @@
         <v>339</v>
       </c>
       <c r="O21" t="n">
-        <v>1898</v>
+        <v>1776</v>
       </c>
       <c r="P21" t="n">
-        <v>1534</v>
+        <v>1427</v>
       </c>
       <c r="Q21" t="n">
-        <v>1386</v>
+        <v>1284</v>
       </c>
       <c r="R21" t="n">
-        <v>1000</v>
+        <v>924</v>
       </c>
       <c r="S21" t="n">
-        <v>722</v>
+        <v>662</v>
       </c>
       <c r="T21" t="n">
-        <v>321</v>
+        <v>284</v>
       </c>
       <c r="U21" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="V21" t="n">
         <v>4042</v>
@@ -21494,25 +21494,25 @@
         <v>55</v>
       </c>
       <c r="O22" t="n">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="P22" t="n">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="Q22" t="n">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="R22" t="n">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="S22" t="n">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="T22" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="U22" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="V22" t="n">
         <v>567</v>
@@ -21578,25 +21578,25 @@
         <v>1100</v>
       </c>
       <c r="O23" t="n">
-        <v>6986</v>
+        <v>6601</v>
       </c>
       <c r="P23" t="n">
-        <v>5976</v>
+        <v>5615</v>
       </c>
       <c r="Q23" t="n">
-        <v>5565</v>
+        <v>5217</v>
       </c>
       <c r="R23" t="n">
-        <v>4332</v>
+        <v>4014</v>
       </c>
       <c r="S23" t="n">
-        <v>3296</v>
+        <v>3023</v>
       </c>
       <c r="T23" t="n">
-        <v>1662</v>
+        <v>1479</v>
       </c>
       <c r="U23" t="n">
-        <v>429</v>
+        <v>360</v>
       </c>
       <c r="V23" t="n">
         <v>13192</v>
@@ -22418,22 +22418,22 @@
         <v>22</v>
       </c>
       <c r="O33" t="n">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="P33" t="n">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="Q33" t="n">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="R33" t="n">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="S33" t="n">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="T33" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="U33" t="n">
         <v>10</v>
@@ -22502,25 +22502,25 @@
         <v>21</v>
       </c>
       <c r="O34" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="P34" t="n">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="Q34" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="R34" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="S34" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="T34" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="U34" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V34" t="n">
         <v>168</v>
@@ -22838,22 +22838,22 @@
         <v>10</v>
       </c>
       <c r="O38" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="P38" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="Q38" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="R38" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="S38" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="T38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U38" t="n">
         <v>2</v>
@@ -22922,25 +22922,25 @@
         <v>70</v>
       </c>
       <c r="O39" t="n">
-        <v>472</v>
+        <v>429</v>
       </c>
       <c r="P39" t="n">
-        <v>402</v>
+        <v>361</v>
       </c>
       <c r="Q39" t="n">
-        <v>381</v>
+        <v>340</v>
       </c>
       <c r="R39" t="n">
-        <v>316</v>
+        <v>276</v>
       </c>
       <c r="S39" t="n">
-        <v>263</v>
+        <v>227</v>
       </c>
       <c r="T39" t="n">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="U39" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="V39" t="n">
         <v>765</v>
@@ -23006,22 +23006,22 @@
         <v>8</v>
       </c>
       <c r="O40" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="P40" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="Q40" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="R40" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="S40" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="T40" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U40" t="n">
         <v>3</v>
@@ -23426,22 +23426,22 @@
         <v>1</v>
       </c>
       <c r="O45" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P45" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q45" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="R45" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S45" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="T45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U45" t="n">
         <v>1</v>
@@ -23510,25 +23510,25 @@
         <v>12</v>
       </c>
       <c r="O46" t="n">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="P46" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="Q46" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="R46" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="S46" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="T46" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="U46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V46" t="n">
         <v>220</v>
@@ -23762,25 +23762,25 @@
         <v>21</v>
       </c>
       <c r="O49" t="n">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="P49" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="Q49" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="R49" t="n">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="S49" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="T49" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="U49" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="V49" t="n">
         <v>117</v>
@@ -23930,22 +23930,22 @@
         <v>19</v>
       </c>
       <c r="O51" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="P51" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="Q51" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="R51" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="S51" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="T51" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="U51" t="n">
         <v>5</v>
@@ -24098,25 +24098,25 @@
         <v>64</v>
       </c>
       <c r="O53" t="n">
-        <v>652</v>
+        <v>635</v>
       </c>
       <c r="P53" t="n">
-        <v>567</v>
+        <v>552</v>
       </c>
       <c r="Q53" t="n">
-        <v>527</v>
+        <v>513</v>
       </c>
       <c r="R53" t="n">
-        <v>433</v>
+        <v>420</v>
       </c>
       <c r="S53" t="n">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="T53" t="n">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="U53" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="V53" t="n">
         <v>1191</v>
@@ -24434,25 +24434,25 @@
         <v>20</v>
       </c>
       <c r="O57" t="n">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="P57" t="n">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="Q57" t="n">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="R57" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="S57" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="T57" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="U57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V57" t="n">
         <v>413</v>
@@ -24518,22 +24518,22 @@
         <v>22</v>
       </c>
       <c r="O58" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="P58" t="n">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="Q58" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="R58" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="S58" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="T58" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="U58" t="n">
         <v>9</v>
@@ -25190,25 +25190,25 @@
         <v>42</v>
       </c>
       <c r="O66" t="n">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="P66" t="n">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="Q66" t="n">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="R66" t="n">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="S66" t="n">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="T66" t="n">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="U66" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="V66" t="n">
         <v>564</v>
@@ -25274,19 +25274,19 @@
         <v>16</v>
       </c>
       <c r="O67" t="n">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="P67" t="n">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="Q67" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="R67" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="S67" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T67" t="n">
         <v>34</v>
@@ -25610,22 +25610,22 @@
         <v>17</v>
       </c>
       <c r="O71" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="P71" t="n">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="Q71" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="R71" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="S71" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="T71" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="U71" t="n">
         <v>1</v>
@@ -25862,19 +25862,19 @@
         <v>5</v>
       </c>
       <c r="O74" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T74" t="n">
         <v>0</v>
@@ -26408,22 +26408,22 @@
         <v>7</v>
       </c>
       <c r="O4" t="n">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="P4" t="n">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Q4" t="n">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="R4" t="n">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="S4" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="T4" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="U4" t="n">
         <v>8</v>
@@ -26492,19 +26492,19 @@
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="R5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T5" t="n">
         <v>4</v>
@@ -26576,22 +26576,22 @@
         <v>4032</v>
       </c>
       <c r="O6" t="n">
-        <v>4646</v>
+        <v>4502</v>
       </c>
       <c r="P6" t="n">
-        <v>2464</v>
+        <v>2372</v>
       </c>
       <c r="Q6" t="n">
-        <v>1951</v>
+        <v>1870</v>
       </c>
       <c r="R6" t="n">
-        <v>953</v>
+        <v>900</v>
       </c>
       <c r="S6" t="n">
-        <v>416</v>
+        <v>387</v>
       </c>
       <c r="T6" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="U6" t="n">
         <v>4</v>
@@ -26744,22 +26744,22 @@
         <v>931</v>
       </c>
       <c r="O8" t="n">
-        <v>508</v>
+        <v>440</v>
       </c>
       <c r="P8" t="n">
-        <v>328</v>
+        <v>281</v>
       </c>
       <c r="Q8" t="n">
-        <v>276</v>
+        <v>229</v>
       </c>
       <c r="R8" t="n">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="S8" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="T8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U8" t="n">
         <v>1</v>
@@ -26912,13 +26912,13 @@
         <v>50</v>
       </c>
       <c r="O10" t="n">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="P10" t="n">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="Q10" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="R10" t="n">
         <v>57</v>
@@ -27080,22 +27080,22 @@
         <v>3998</v>
       </c>
       <c r="O12" t="n">
-        <v>5630</v>
+        <v>5456</v>
       </c>
       <c r="P12" t="n">
-        <v>2665</v>
+        <v>2570</v>
       </c>
       <c r="Q12" t="n">
-        <v>1981</v>
+        <v>1902</v>
       </c>
       <c r="R12" t="n">
-        <v>817</v>
+        <v>782</v>
       </c>
       <c r="S12" t="n">
-        <v>317</v>
+        <v>304</v>
       </c>
       <c r="T12" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -27164,19 +27164,19 @@
         <v>1124</v>
       </c>
       <c r="O13" t="n">
-        <v>3027</v>
+        <v>2956</v>
       </c>
       <c r="P13" t="n">
-        <v>1109</v>
+        <v>1070</v>
       </c>
       <c r="Q13" t="n">
-        <v>757</v>
+        <v>728</v>
       </c>
       <c r="R13" t="n">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="S13" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="T13" t="n">
         <v>8</v>
@@ -27584,19 +27584,19 @@
         <v>5</v>
       </c>
       <c r="O18" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P18" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q18" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="R18" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S18" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="T18" t="n">
         <v>46</v>
@@ -28634,22 +28634,22 @@
         <v>3</v>
       </c>
       <c r="O12" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P12" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Q12" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R12" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="S12" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U12" t="n">
         <v>2</v>
@@ -29558,16 +29558,16 @@
         <v>8</v>
       </c>
       <c r="O23" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P23" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q23" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R23" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S23" t="n">
         <v>22</v>
@@ -29978,25 +29978,25 @@
         <v>8</v>
       </c>
       <c r="O28" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="P28" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="Q28" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="R28" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="S28" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="T28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="U28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V28" t="n">
         <v>287</v>
@@ -32330,19 +32330,19 @@
         <v>59</v>
       </c>
       <c r="O56" t="n">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="P56" t="n">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Q56" t="n">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="R56" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="S56" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="T56" t="n">
         <v>26</v>
@@ -32582,25 +32582,25 @@
         <v>55</v>
       </c>
       <c r="O59" t="n">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="P59" t="n">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="Q59" t="n">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="R59" t="n">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="S59" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="T59" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="U59" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="V59" t="n">
         <v>875</v>
@@ -32666,22 +32666,22 @@
         <v>12</v>
       </c>
       <c r="O60" t="n">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="P60" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="Q60" t="n">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="R60" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="S60" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T60" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U60" t="n">
         <v>14</v>
@@ -34976,22 +34976,22 @@
         <v>5</v>
       </c>
       <c r="O12" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="P12" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="Q12" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -35396,7 +35396,7 @@
         <v>141</v>
       </c>
       <c r="O17" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P17" t="n">
         <v>150</v>
@@ -37244,16 +37244,16 @@
         <v>114</v>
       </c>
       <c r="O39" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P39" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q39" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R39" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="S39" t="n">
         <v>13</v>
@@ -38378,19 +38378,19 @@
         <v>23</v>
       </c>
       <c r="O2" t="n">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="P2" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="Q2" t="n">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="R2" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="S2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="T2" t="n">
         <v>19</v>
@@ -38546,16 +38546,16 @@
         <v>17</v>
       </c>
       <c r="O4" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="P4" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Q4" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="S4" t="n">
         <v>12</v>
@@ -38798,25 +38798,25 @@
         <v>591</v>
       </c>
       <c r="O7" t="n">
-        <v>5699</v>
+        <v>5630</v>
       </c>
       <c r="P7" t="n">
-        <v>3421</v>
+        <v>3366</v>
       </c>
       <c r="Q7" t="n">
-        <v>2732</v>
+        <v>2682</v>
       </c>
       <c r="R7" t="n">
-        <v>1258</v>
+        <v>1227</v>
       </c>
       <c r="S7" t="n">
-        <v>651</v>
+        <v>628</v>
       </c>
       <c r="T7" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="U7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V7" t="n">
         <v>27977</v>
@@ -39050,19 +39050,19 @@
         <v>153</v>
       </c>
       <c r="O10" t="n">
-        <v>3093</v>
+        <v>3060</v>
       </c>
       <c r="P10" t="n">
-        <v>1671</v>
+        <v>1648</v>
       </c>
       <c r="Q10" t="n">
-        <v>1299</v>
+        <v>1280</v>
       </c>
       <c r="R10" t="n">
-        <v>509</v>
+        <v>499</v>
       </c>
       <c r="S10" t="n">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="T10" t="n">
         <v>39</v>
@@ -39134,13 +39134,13 @@
         <v>39</v>
       </c>
       <c r="O11" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="P11" t="n">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="Q11" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="R11" t="n">
         <v>46</v>
@@ -39218,22 +39218,22 @@
         <v>76</v>
       </c>
       <c r="O12" t="n">
-        <v>1146</v>
+        <v>1143</v>
       </c>
       <c r="P12" t="n">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="Q12" t="n">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="R12" t="n">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="S12" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="T12" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="U12" t="n">
         <v>2</v>
@@ -39302,7 +39302,7 @@
         <v>7</v>
       </c>
       <c r="O13" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P13" t="n">
         <v>14</v>
@@ -39386,25 +39386,25 @@
         <v>374</v>
       </c>
       <c r="O14" t="n">
-        <v>3840</v>
+        <v>3786</v>
       </c>
       <c r="P14" t="n">
-        <v>2091</v>
+        <v>2059</v>
       </c>
       <c r="Q14" t="n">
-        <v>1620</v>
+        <v>1595</v>
       </c>
       <c r="R14" t="n">
-        <v>689</v>
+        <v>675</v>
       </c>
       <c r="S14" t="n">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="T14" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="U14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V14" t="n">
         <v>27838</v>
@@ -39470,19 +39470,19 @@
         <v>100</v>
       </c>
       <c r="O15" t="n">
-        <v>546</v>
+        <v>537</v>
       </c>
       <c r="P15" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="Q15" t="n">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="R15" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="S15" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="T15" t="n">
         <v>11</v>
@@ -40352,22 +40352,22 @@
         <v>10</v>
       </c>
       <c r="O8" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="P8" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="Q8" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="R8" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S8" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="T8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U8" t="n">
         <v>4</v>
@@ -41360,25 +41360,25 @@
         <v>19</v>
       </c>
       <c r="O20" t="n">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="P20" t="n">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="Q20" t="n">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="R20" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="S20" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="T20" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="U20" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V20" t="n">
         <v>495</v>
@@ -41444,22 +41444,22 @@
         <v>9</v>
       </c>
       <c r="O21" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P21" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q21" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="R21" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S21" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T21" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U21" t="n">
         <v>7</v>
@@ -41528,25 +41528,25 @@
         <v>176</v>
       </c>
       <c r="O22" t="n">
-        <v>2989</v>
+        <v>2974</v>
       </c>
       <c r="P22" t="n">
-        <v>2283</v>
+        <v>2268</v>
       </c>
       <c r="Q22" t="n">
-        <v>2057</v>
+        <v>2042</v>
       </c>
       <c r="R22" t="n">
-        <v>1453</v>
+        <v>1440</v>
       </c>
       <c r="S22" t="n">
-        <v>1071</v>
+        <v>1058</v>
       </c>
       <c r="T22" t="n">
-        <v>553</v>
+        <v>544</v>
       </c>
       <c r="U22" t="n">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="V22" t="n">
         <v>6934</v>
@@ -41696,25 +41696,25 @@
         <v>174</v>
       </c>
       <c r="O24" t="n">
-        <v>1283</v>
+        <v>1268</v>
       </c>
       <c r="P24" t="n">
-        <v>1018</v>
+        <v>1004</v>
       </c>
       <c r="Q24" t="n">
-        <v>910</v>
+        <v>897</v>
       </c>
       <c r="R24" t="n">
-        <v>608</v>
+        <v>597</v>
       </c>
       <c r="S24" t="n">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="T24" t="n">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="U24" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="V24" t="n">
         <v>3129</v>
@@ -41948,16 +41948,16 @@
         <v>327</v>
       </c>
       <c r="O27" t="n">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="P27" t="n">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="Q27" t="n">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="R27" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="S27" t="n">
         <v>52</v>
@@ -42200,25 +42200,25 @@
         <v>7820</v>
       </c>
       <c r="O30" t="n">
-        <v>42279</v>
+        <v>41819</v>
       </c>
       <c r="P30" t="n">
-        <v>23477</v>
+        <v>23134</v>
       </c>
       <c r="Q30" t="n">
-        <v>18494</v>
+        <v>18185</v>
       </c>
       <c r="R30" t="n">
-        <v>9176</v>
+        <v>8957</v>
       </c>
       <c r="S30" t="n">
-        <v>5310</v>
+        <v>5154</v>
       </c>
       <c r="T30" t="n">
-        <v>1693</v>
+        <v>1614</v>
       </c>
       <c r="U30" t="n">
-        <v>375</v>
+        <v>357</v>
       </c>
       <c r="V30" t="n">
         <v>217988</v>
@@ -42284,22 +42284,22 @@
         <v>334</v>
       </c>
       <c r="O31" t="n">
-        <v>1247</v>
+        <v>1243</v>
       </c>
       <c r="P31" t="n">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="Q31" t="n">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="R31" t="n">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="S31" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="T31" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="U31" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Re run after changind deduplication step Flix and WB
</commit_message>
<xml_diff>
--- a/summary_stats/chuuchuu_summary_2025_01.xlsx
+++ b/summary_stats/chuuchuu_summary_2025_01.xlsx
@@ -17554,7 +17554,7 @@
         </is>
       </c>
       <c r="J217" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K217" t="n">
         <v>0</v>
@@ -17587,7 +17587,7 @@
         <v>1</v>
       </c>
       <c r="U217" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="218">

</xml_diff>